<commit_message>
EVT-004: Marine AV vendor research Phase 1 & 2 complete - 5 emails sent to verified contacts
</commit_message>
<xml_diff>
--- a/EVT-004_Photography_Vendors_Phase1.xlsx
+++ b/EVT-004_Photography_Vendors_Phase1.xlsx
@@ -603,14 +603,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>19c320e4cfb2d5c3</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
           <t>SF &amp; LV based, corporate events, conferences, 24hr delivery</t>
@@ -663,14 +675,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>19c320e713dac851</t>
+        </is>
+      </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
           <t>16+ years exp, Google/LinkedIn/Salesforce clients, high-capacity conferences</t>
@@ -723,14 +747,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>19c320e9c8c45d35</t>
+        </is>
+      </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Boutique agency, trusted by top brands, nationwide coverage</t>
@@ -783,14 +819,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>19c320ea003c95f6</t>
+        </is>
+      </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Award-winning, 25,000+ attendee conferences, SF Bay Area &amp; worldwide</t>
@@ -843,14 +891,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>19c320ec52019b9e</t>
+        </is>
+      </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Corporate events, conferences, large-scale summits, brand activations</t>
@@ -899,14 +959,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>19c320ec912ea8cf</t>
+        </is>
+      </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Team of photographers, 500+ events, SF native, tech companies/galas</t>
@@ -959,14 +1031,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>19c320eeb810ecef</t>
+        </is>
+      </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
           <t>12+ years exp, Google/PayPal/Salesforce, 24hr delivery, fully insured</t>
@@ -1019,14 +1103,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>19c320eef91d94f4</t>
+        </is>
+      </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
           <t>Team-based, PR/corporate/marketing specialization, major SF events</t>
@@ -1075,14 +1171,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>19c320f13efd4f0c</t>
+        </is>
+      </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
           <t>Documentary style, conferences/retreats/parties, video services, photobooth</t>
@@ -1135,14 +1243,26 @@
           <t>2026-02-06</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>00:23 PST</t>
+        </is>
+      </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Research Complete</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr"/>
+          <t>Email Sent</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>19c320f17ea3d64b</t>
+        </is>
+      </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
           <t>25 years event marketing, 16 years photography, SF Bay &amp; Vegas, conferences/galas</t>

</xml_diff>